<commit_message>
XRO forecast update 2026-08
</commit_message>
<xml_diff>
--- a/content/climate/XRO/XRO_ENSO_fcst.xlsx
+++ b/content/climate/XRO/XRO_ENSO_fcst.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>2023-01</t>
   </si>
@@ -143,10 +143,13 @@
     <t>2026-06</t>
   </si>
   <si>
+    <t>2026-07</t>
+  </si>
+  <si>
     <t>Readme</t>
   </si>
   <si>
-    <t>Extended nonlinear recharge oscillator (XRO) ENSO forecast (Zhao et al. 2024)</t>
+    <t>Extended nonlinear recharge oscillator (XRO) Nino34 forecast</t>
   </si>
   <si>
     <t>Reference: Zhao et al. (2024), Nature</t>
@@ -517,7 +520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U43"/>
+  <dimension ref="A1:U44"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="21" width="10.7109375" style="1" customWidth="1"/>
@@ -525,7 +528,7 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B1" s="2">
         <v>0</v>
@@ -2936,61 +2939,61 @@
         <v>-0.5590000000000001</v>
       </c>
       <c r="C38" s="1">
-        <v>-0.452</v>
+        <v>-0.447</v>
       </c>
       <c r="D38" s="1">
-        <v>-0.302</v>
+        <v>-0.303</v>
       </c>
       <c r="E38" s="1">
-        <v>-0.201</v>
+        <v>-0.202</v>
       </c>
       <c r="F38" s="1">
-        <v>-0.081</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="G38" s="1">
-        <v>0.079</v>
+        <v>0.113</v>
       </c>
       <c r="H38" s="1">
-        <v>0.278</v>
+        <v>0.314</v>
       </c>
       <c r="I38" s="1">
-        <v>0.477</v>
+        <v>0.475</v>
       </c>
       <c r="J38" s="1">
-        <v>0.655</v>
+        <v>0.611</v>
       </c>
       <c r="K38" s="1">
-        <v>0.83</v>
+        <v>0.769</v>
       </c>
       <c r="L38" s="1">
-        <v>1.005</v>
+        <v>0.947</v>
       </c>
       <c r="M38" s="1">
-        <v>1.147</v>
+        <v>1.118</v>
       </c>
       <c r="N38" s="1">
-        <v>1.195</v>
+        <v>1.18</v>
       </c>
       <c r="O38" s="1">
-        <v>1.125</v>
+        <v>1.103</v>
       </c>
       <c r="P38" s="1">
-        <v>0.97</v>
+        <v>0.9389999999999999</v>
       </c>
       <c r="Q38" s="1">
-        <v>0.769</v>
+        <v>0.749</v>
       </c>
       <c r="R38" s="1">
-        <v>0.5679999999999999</v>
+        <v>0.58</v>
       </c>
       <c r="S38" s="1">
-        <v>0.399</v>
+        <v>0.423</v>
       </c>
       <c r="T38" s="1">
-        <v>0.239</v>
+        <v>0.294</v>
       </c>
       <c r="U38" s="1">
-        <v>0.117</v>
+        <v>0.218</v>
       </c>
     </row>
     <row r="39" spans="1:21">
@@ -3001,10 +3004,10 @@
         <v>-0.273</v>
       </c>
       <c r="C39" s="1">
-        <v>-0.212</v>
+        <v>-0.2</v>
       </c>
       <c r="D39" s="1">
-        <v>-0.109</v>
+        <v>-0.09</v>
       </c>
       <c r="E39" s="1">
         <v>0.043</v>
@@ -3013,49 +3016,49 @@
         <v>0.247</v>
       </c>
       <c r="G39" s="1">
-        <v>0.477</v>
+        <v>0.493</v>
       </c>
       <c r="H39" s="1">
-        <v>0.717</v>
+        <v>0.729</v>
       </c>
       <c r="I39" s="1">
-        <v>0.924</v>
+        <v>0.946</v>
       </c>
       <c r="J39" s="1">
-        <v>1.112</v>
+        <v>1.179</v>
       </c>
       <c r="K39" s="1">
-        <v>1.298</v>
+        <v>1.424</v>
       </c>
       <c r="L39" s="1">
-        <v>1.43</v>
+        <v>1.605</v>
       </c>
       <c r="M39" s="1">
-        <v>1.451</v>
+        <v>1.627</v>
       </c>
       <c r="N39" s="1">
-        <v>1.352</v>
+        <v>1.498</v>
       </c>
       <c r="O39" s="1">
-        <v>1.156</v>
+        <v>1.267</v>
       </c>
       <c r="P39" s="1">
-        <v>0.91</v>
+        <v>0.989</v>
       </c>
       <c r="Q39" s="1">
-        <v>0.646</v>
+        <v>0.704</v>
       </c>
       <c r="R39" s="1">
-        <v>0.391</v>
+        <v>0.414</v>
       </c>
       <c r="S39" s="1">
-        <v>0.171</v>
+        <v>0.186</v>
       </c>
       <c r="T39" s="1">
-        <v>0.027</v>
+        <v>0.062</v>
       </c>
       <c r="U39" s="1">
-        <v>-0.03</v>
+        <v>-0.003</v>
       </c>
     </row>
     <row r="40" spans="1:21">
@@ -3066,61 +3069,61 @@
         <v>-0.008</v>
       </c>
       <c r="C40" s="1">
-        <v>0.064</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="D40" s="1">
-        <v>0.247</v>
+        <v>0.29</v>
       </c>
       <c r="E40" s="1">
-        <v>0.52</v>
+        <v>0.536</v>
       </c>
       <c r="F40" s="1">
-        <v>0.838</v>
+        <v>0.819</v>
       </c>
       <c r="G40" s="1">
-        <v>1.128</v>
+        <v>1.121</v>
       </c>
       <c r="H40" s="1">
-        <v>1.417</v>
+        <v>1.419</v>
       </c>
       <c r="I40" s="1">
-        <v>1.723</v>
+        <v>1.745</v>
       </c>
       <c r="J40" s="1">
-        <v>2</v>
+        <v>2.061</v>
       </c>
       <c r="K40" s="1">
-        <v>2.189</v>
+        <v>2.27</v>
       </c>
       <c r="L40" s="1">
-        <v>2.218</v>
+        <v>2.28</v>
       </c>
       <c r="M40" s="1">
-        <v>2.063</v>
+        <v>2.088</v>
       </c>
       <c r="N40" s="1">
-        <v>1.744</v>
+        <v>1.754</v>
       </c>
       <c r="O40" s="1">
-        <v>1.348</v>
+        <v>1.347</v>
       </c>
       <c r="P40" s="1">
-        <v>0.949</v>
+        <v>0.93</v>
       </c>
       <c r="Q40" s="1">
-        <v>0.554</v>
+        <v>0.533</v>
       </c>
       <c r="R40" s="1">
-        <v>0.21</v>
+        <v>0.203</v>
       </c>
       <c r="S40" s="1">
-        <v>0.001</v>
+        <v>-0.002</v>
       </c>
       <c r="T40" s="1">
-        <v>-0.099</v>
+        <v>-0.094</v>
       </c>
       <c r="U40" s="1">
-        <v>-0.155</v>
+        <v>-0.146</v>
       </c>
     </row>
     <row r="41" spans="1:21">
@@ -3131,61 +3134,61 @@
         <v>0.452</v>
       </c>
       <c r="C41" s="1">
-        <v>0.585</v>
+        <v>0.597</v>
       </c>
       <c r="D41" s="1">
-        <v>0.885</v>
+        <v>0.912</v>
       </c>
       <c r="E41" s="1">
-        <v>1.311</v>
+        <v>1.304</v>
       </c>
       <c r="F41" s="1">
-        <v>1.797</v>
+        <v>1.731</v>
       </c>
       <c r="G41" s="1">
-        <v>2.288</v>
+        <v>2.182</v>
       </c>
       <c r="H41" s="1">
-        <v>2.757</v>
+        <v>2.614</v>
       </c>
       <c r="I41" s="1">
-        <v>3.132</v>
+        <v>2.969</v>
       </c>
       <c r="J41" s="1">
-        <v>3.349</v>
+        <v>3.186</v>
       </c>
       <c r="K41" s="1">
-        <v>3.365</v>
+        <v>3.203</v>
       </c>
       <c r="L41" s="1">
-        <v>3.144</v>
+        <v>2.972</v>
       </c>
       <c r="M41" s="1">
-        <v>2.645</v>
+        <v>2.488</v>
       </c>
       <c r="N41" s="1">
-        <v>1.96</v>
+        <v>1.844</v>
       </c>
       <c r="O41" s="1">
-        <v>1.264</v>
+        <v>1.21</v>
       </c>
       <c r="P41" s="1">
-        <v>0.627</v>
+        <v>0.62</v>
       </c>
       <c r="Q41" s="1">
-        <v>0.091</v>
+        <v>0.13</v>
       </c>
       <c r="R41" s="1">
-        <v>-0.238</v>
+        <v>-0.155</v>
       </c>
       <c r="S41" s="1">
-        <v>-0.377</v>
+        <v>-0.284</v>
       </c>
       <c r="T41" s="1">
-        <v>-0.464</v>
+        <v>-0.382</v>
       </c>
       <c r="U41" s="1">
-        <v>-0.5620000000000001</v>
+        <v>-0.499</v>
       </c>
     </row>
     <row r="42" spans="1:21">
@@ -3196,61 +3199,61 @@
         <v>1.04</v>
       </c>
       <c r="C42" s="1">
-        <v>1.22</v>
+        <v>1.235</v>
       </c>
       <c r="D42" s="1">
-        <v>1.599</v>
+        <v>1.614</v>
       </c>
       <c r="E42" s="1">
-        <v>2.056</v>
+        <v>2.037</v>
       </c>
       <c r="F42" s="1">
-        <v>2.528</v>
+        <v>2.506</v>
       </c>
       <c r="G42" s="1">
-        <v>2.926</v>
+        <v>2.961</v>
       </c>
       <c r="H42" s="1">
-        <v>3.175</v>
+        <v>3.248</v>
       </c>
       <c r="I42" s="1">
-        <v>3.272</v>
+        <v>3.351</v>
       </c>
       <c r="J42" s="1">
-        <v>3.207</v>
+        <v>3.27</v>
       </c>
       <c r="K42" s="1">
-        <v>2.931</v>
+        <v>2.981</v>
       </c>
       <c r="L42" s="1">
-        <v>2.421</v>
+        <v>2.479</v>
       </c>
       <c r="M42" s="1">
-        <v>1.772</v>
+        <v>1.84</v>
       </c>
       <c r="N42" s="1">
-        <v>1.112</v>
+        <v>1.169</v>
       </c>
       <c r="O42" s="1">
-        <v>0.5</v>
+        <v>0.538</v>
       </c>
       <c r="P42" s="1">
-        <v>0.001</v>
+        <v>0.034</v>
       </c>
       <c r="Q42" s="1">
-        <v>-0.27</v>
+        <v>-0.242</v>
       </c>
       <c r="R42" s="1">
-        <v>-0.381</v>
+        <v>-0.346</v>
       </c>
       <c r="S42" s="1">
-        <v>-0.454</v>
+        <v>-0.414</v>
       </c>
       <c r="T42" s="1">
-        <v>-0.5570000000000001</v>
+        <v>-0.511</v>
       </c>
       <c r="U42" s="1">
-        <v>-0.67</v>
+        <v>-0.61</v>
       </c>
     </row>
     <row r="43" spans="1:21">
@@ -3261,61 +3264,126 @@
         <v>1.526</v>
       </c>
       <c r="C43" s="1">
-        <v>1.843</v>
+        <v>1.842</v>
       </c>
       <c r="D43" s="1">
-        <v>2.462</v>
+        <v>2.44</v>
       </c>
       <c r="E43" s="1">
-        <v>3.106</v>
+        <v>3.045</v>
       </c>
       <c r="F43" s="1">
-        <v>3.591</v>
+        <v>3.506</v>
       </c>
       <c r="G43" s="1">
-        <v>3.792</v>
+        <v>3.705</v>
       </c>
       <c r="H43" s="1">
-        <v>3.78</v>
+        <v>3.699</v>
       </c>
       <c r="I43" s="1">
-        <v>3.625</v>
+        <v>3.54</v>
       </c>
       <c r="J43" s="1">
-        <v>3.295</v>
+        <v>3.196</v>
       </c>
       <c r="K43" s="1">
-        <v>2.728</v>
+        <v>2.624</v>
       </c>
       <c r="L43" s="1">
-        <v>1.959</v>
+        <v>1.905</v>
       </c>
       <c r="M43" s="1">
-        <v>1.157</v>
+        <v>1.142</v>
       </c>
       <c r="N43" s="1">
-        <v>0.394</v>
+        <v>0.409</v>
       </c>
       <c r="O43" s="1">
-        <v>-0.198</v>
+        <v>-0.167</v>
       </c>
       <c r="P43" s="1">
-        <v>-0.491</v>
+        <v>-0.466</v>
       </c>
       <c r="Q43" s="1">
-        <v>-0.585</v>
+        <v>-0.5620000000000001</v>
       </c>
       <c r="R43" s="1">
-        <v>-0.665</v>
+        <v>-0.644</v>
       </c>
       <c r="S43" s="1">
-        <v>-0.8179999999999999</v>
+        <v>-0.8090000000000001</v>
       </c>
       <c r="T43" s="1">
-        <v>-0.985</v>
+        <v>-0.993</v>
       </c>
       <c r="U43" s="1">
-        <v>-1.014</v>
+        <v>-1.023</v>
+      </c>
+    </row>
+    <row r="44" spans="1:21">
+      <c r="A44" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B44" s="1">
+        <v>2.085</v>
+      </c>
+      <c r="C44" s="1">
+        <v>2.565</v>
+      </c>
+      <c r="D44" s="1">
+        <v>3.451</v>
+      </c>
+      <c r="E44" s="1">
+        <v>4.151</v>
+      </c>
+      <c r="F44" s="1">
+        <v>4.449</v>
+      </c>
+      <c r="G44" s="1">
+        <v>4.458</v>
+      </c>
+      <c r="H44" s="1">
+        <v>4.312</v>
+      </c>
+      <c r="I44" s="1">
+        <v>3.936</v>
+      </c>
+      <c r="J44" s="1">
+        <v>3.218</v>
+      </c>
+      <c r="K44" s="1">
+        <v>2.279</v>
+      </c>
+      <c r="L44" s="1">
+        <v>1.313</v>
+      </c>
+      <c r="M44" s="1">
+        <v>0.395</v>
+      </c>
+      <c r="N44" s="1">
+        <v>-0.314</v>
+      </c>
+      <c r="O44" s="1">
+        <v>-0.65</v>
+      </c>
+      <c r="P44" s="1">
+        <v>-0.742</v>
+      </c>
+      <c r="Q44" s="1">
+        <v>-0.8100000000000001</v>
+      </c>
+      <c r="R44" s="1">
+        <v>-0.995</v>
+      </c>
+      <c r="S44" s="1">
+        <v>-1.233</v>
+      </c>
+      <c r="T44" s="1">
+        <v>-1.273</v>
+      </c>
+      <c r="U44" s="1">
+        <v>-1.085</v>
       </c>
     </row>
   </sheetData>
@@ -3330,22 +3398,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
XRO Forecast From 2026-09
</commit_message>
<xml_diff>
--- a/content/climate/XRO/XRO_ENSO_fcst.xlsx
+++ b/content/climate/XRO/XRO_ENSO_fcst.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>2023-01</t>
   </si>
@@ -144,6 +144,9 @@
   </si>
   <si>
     <t>2026-07</t>
+  </si>
+  <si>
+    <t>2026-08</t>
   </si>
   <si>
     <t>Readme</t>
@@ -520,7 +523,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U44"/>
+  <dimension ref="A1:U45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="21" width="10.7109375" style="1" customWidth="1"/>
@@ -528,7 +531,7 @@
   <sheetData>
     <row r="1" spans="1:21">
       <c r="A1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B1" s="2">
         <v>0</v>
@@ -2939,61 +2942,61 @@
         <v>-0.5590000000000001</v>
       </c>
       <c r="C38" s="1">
-        <v>-0.447</v>
+        <v>-0.452</v>
       </c>
       <c r="D38" s="1">
-        <v>-0.303</v>
+        <v>-0.309</v>
       </c>
       <c r="E38" s="1">
-        <v>-0.202</v>
+        <v>-0.192</v>
       </c>
       <c r="F38" s="1">
-        <v>-0.07000000000000001</v>
+        <v>-0.029</v>
       </c>
       <c r="G38" s="1">
-        <v>0.113</v>
+        <v>0.18</v>
       </c>
       <c r="H38" s="1">
-        <v>0.314</v>
+        <v>0.4</v>
       </c>
       <c r="I38" s="1">
-        <v>0.475</v>
+        <v>0.588</v>
       </c>
       <c r="J38" s="1">
-        <v>0.611</v>
+        <v>0.759</v>
       </c>
       <c r="K38" s="1">
-        <v>0.769</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="L38" s="1">
-        <v>0.947</v>
+        <v>1.118</v>
       </c>
       <c r="M38" s="1">
-        <v>1.118</v>
+        <v>1.242</v>
       </c>
       <c r="N38" s="1">
-        <v>1.18</v>
+        <v>1.245</v>
       </c>
       <c r="O38" s="1">
-        <v>1.103</v>
+        <v>1.137</v>
       </c>
       <c r="P38" s="1">
-        <v>0.9389999999999999</v>
+        <v>0.957</v>
       </c>
       <c r="Q38" s="1">
-        <v>0.749</v>
+        <v>0.741</v>
       </c>
       <c r="R38" s="1">
-        <v>0.58</v>
+        <v>0.538</v>
       </c>
       <c r="S38" s="1">
-        <v>0.423</v>
+        <v>0.342</v>
       </c>
       <c r="T38" s="1">
-        <v>0.294</v>
+        <v>0.172</v>
       </c>
       <c r="U38" s="1">
-        <v>0.218</v>
+        <v>0.058</v>
       </c>
     </row>
     <row r="39" spans="1:21">
@@ -3004,61 +3007,61 @@
         <v>-0.273</v>
       </c>
       <c r="C39" s="1">
-        <v>-0.2</v>
+        <v>-0.208</v>
       </c>
       <c r="D39" s="1">
-        <v>-0.09</v>
+        <v>-0.08500000000000001</v>
       </c>
       <c r="E39" s="1">
-        <v>0.043</v>
+        <v>0.078</v>
       </c>
       <c r="F39" s="1">
-        <v>0.247</v>
+        <v>0.294</v>
       </c>
       <c r="G39" s="1">
-        <v>0.493</v>
+        <v>0.527</v>
       </c>
       <c r="H39" s="1">
-        <v>0.729</v>
+        <v>0.771</v>
       </c>
       <c r="I39" s="1">
-        <v>0.946</v>
+        <v>0.993</v>
       </c>
       <c r="J39" s="1">
-        <v>1.179</v>
+        <v>1.206</v>
       </c>
       <c r="K39" s="1">
-        <v>1.424</v>
+        <v>1.419</v>
       </c>
       <c r="L39" s="1">
-        <v>1.605</v>
+        <v>1.579</v>
       </c>
       <c r="M39" s="1">
-        <v>1.627</v>
+        <v>1.624</v>
       </c>
       <c r="N39" s="1">
-        <v>1.498</v>
+        <v>1.488</v>
       </c>
       <c r="O39" s="1">
-        <v>1.267</v>
+        <v>1.252</v>
       </c>
       <c r="P39" s="1">
-        <v>0.989</v>
+        <v>0.983</v>
       </c>
       <c r="Q39" s="1">
-        <v>0.704</v>
+        <v>0.6889999999999999</v>
       </c>
       <c r="R39" s="1">
-        <v>0.414</v>
+        <v>0.423</v>
       </c>
       <c r="S39" s="1">
-        <v>0.186</v>
+        <v>0.211</v>
       </c>
       <c r="T39" s="1">
-        <v>0.062</v>
+        <v>0.08599999999999999</v>
       </c>
       <c r="U39" s="1">
-        <v>-0.003</v>
+        <v>0.031</v>
       </c>
     </row>
     <row r="40" spans="1:21">
@@ -3069,61 +3072,61 @@
         <v>-0.008</v>
       </c>
       <c r="C40" s="1">
-        <v>0.08599999999999999</v>
+        <v>0.073</v>
       </c>
       <c r="D40" s="1">
-        <v>0.29</v>
+        <v>0.278</v>
       </c>
       <c r="E40" s="1">
-        <v>0.536</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="F40" s="1">
-        <v>0.819</v>
+        <v>0.885</v>
       </c>
       <c r="G40" s="1">
-        <v>1.121</v>
+        <v>1.207</v>
       </c>
       <c r="H40" s="1">
-        <v>1.419</v>
+        <v>1.529</v>
       </c>
       <c r="I40" s="1">
-        <v>1.745</v>
+        <v>1.864</v>
       </c>
       <c r="J40" s="1">
-        <v>2.061</v>
+        <v>2.163</v>
       </c>
       <c r="K40" s="1">
-        <v>2.27</v>
+        <v>2.352</v>
       </c>
       <c r="L40" s="1">
-        <v>2.28</v>
+        <v>2.375</v>
       </c>
       <c r="M40" s="1">
-        <v>2.088</v>
+        <v>2.194</v>
       </c>
       <c r="N40" s="1">
-        <v>1.754</v>
+        <v>1.853</v>
       </c>
       <c r="O40" s="1">
-        <v>1.347</v>
+        <v>1.415</v>
       </c>
       <c r="P40" s="1">
-        <v>0.93</v>
+        <v>0.96</v>
       </c>
       <c r="Q40" s="1">
-        <v>0.533</v>
+        <v>0.512</v>
       </c>
       <c r="R40" s="1">
-        <v>0.203</v>
+        <v>0.14</v>
       </c>
       <c r="S40" s="1">
-        <v>-0.002</v>
+        <v>-0.097</v>
       </c>
       <c r="T40" s="1">
-        <v>-0.094</v>
+        <v>-0.224</v>
       </c>
       <c r="U40" s="1">
-        <v>-0.146</v>
+        <v>-0.304</v>
       </c>
     </row>
     <row r="41" spans="1:21">
@@ -3134,61 +3137,61 @@
         <v>0.452</v>
       </c>
       <c r="C41" s="1">
-        <v>0.597</v>
+        <v>0.589</v>
       </c>
       <c r="D41" s="1">
-        <v>0.912</v>
+        <v>0.897</v>
       </c>
       <c r="E41" s="1">
-        <v>1.304</v>
+        <v>1.293</v>
       </c>
       <c r="F41" s="1">
-        <v>1.731</v>
+        <v>1.743</v>
       </c>
       <c r="G41" s="1">
-        <v>2.182</v>
+        <v>2.241</v>
       </c>
       <c r="H41" s="1">
-        <v>2.614</v>
+        <v>2.735</v>
       </c>
       <c r="I41" s="1">
-        <v>2.969</v>
+        <v>3.123</v>
       </c>
       <c r="J41" s="1">
-        <v>3.186</v>
+        <v>3.338</v>
       </c>
       <c r="K41" s="1">
-        <v>3.203</v>
+        <v>3.352</v>
       </c>
       <c r="L41" s="1">
-        <v>2.972</v>
+        <v>3.134</v>
       </c>
       <c r="M41" s="1">
-        <v>2.488</v>
+        <v>2.648</v>
       </c>
       <c r="N41" s="1">
-        <v>1.844</v>
+        <v>1.973</v>
       </c>
       <c r="O41" s="1">
-        <v>1.21</v>
+        <v>1.263</v>
       </c>
       <c r="P41" s="1">
-        <v>0.62</v>
+        <v>0.624</v>
       </c>
       <c r="Q41" s="1">
-        <v>0.13</v>
+        <v>0.143</v>
       </c>
       <c r="R41" s="1">
-        <v>-0.155</v>
+        <v>-0.141</v>
       </c>
       <c r="S41" s="1">
-        <v>-0.284</v>
+        <v>-0.281</v>
       </c>
       <c r="T41" s="1">
-        <v>-0.382</v>
+        <v>-0.372</v>
       </c>
       <c r="U41" s="1">
-        <v>-0.499</v>
+        <v>-0.483</v>
       </c>
     </row>
     <row r="42" spans="1:21">
@@ -3199,61 +3202,61 @@
         <v>1.04</v>
       </c>
       <c r="C42" s="1">
-        <v>1.235</v>
+        <v>1.223</v>
       </c>
       <c r="D42" s="1">
-        <v>1.614</v>
+        <v>1.617</v>
       </c>
       <c r="E42" s="1">
-        <v>2.037</v>
+        <v>2.138</v>
       </c>
       <c r="F42" s="1">
-        <v>2.506</v>
+        <v>2.699</v>
       </c>
       <c r="G42" s="1">
-        <v>2.961</v>
+        <v>3.173</v>
       </c>
       <c r="H42" s="1">
-        <v>3.248</v>
+        <v>3.454</v>
       </c>
       <c r="I42" s="1">
-        <v>3.351</v>
+        <v>3.538</v>
       </c>
       <c r="J42" s="1">
-        <v>3.27</v>
+        <v>3.473</v>
       </c>
       <c r="K42" s="1">
-        <v>2.981</v>
+        <v>3.195</v>
       </c>
       <c r="L42" s="1">
-        <v>2.479</v>
+        <v>2.659</v>
       </c>
       <c r="M42" s="1">
-        <v>1.84</v>
+        <v>1.962</v>
       </c>
       <c r="N42" s="1">
-        <v>1.169</v>
+        <v>1.244</v>
       </c>
       <c r="O42" s="1">
-        <v>0.538</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="P42" s="1">
-        <v>0.034</v>
+        <v>0.004</v>
       </c>
       <c r="Q42" s="1">
-        <v>-0.242</v>
+        <v>-0.317</v>
       </c>
       <c r="R42" s="1">
-        <v>-0.346</v>
+        <v>-0.446</v>
       </c>
       <c r="S42" s="1">
-        <v>-0.414</v>
+        <v>-0.508</v>
       </c>
       <c r="T42" s="1">
-        <v>-0.511</v>
+        <v>-0.618</v>
       </c>
       <c r="U42" s="1">
-        <v>-0.61</v>
+        <v>-0.754</v>
       </c>
     </row>
     <row r="43" spans="1:21">
@@ -3264,61 +3267,61 @@
         <v>1.526</v>
       </c>
       <c r="C43" s="1">
-        <v>1.842</v>
+        <v>1.857</v>
       </c>
       <c r="D43" s="1">
-        <v>2.44</v>
+        <v>2.519</v>
       </c>
       <c r="E43" s="1">
-        <v>3.045</v>
+        <v>3.199</v>
       </c>
       <c r="F43" s="1">
-        <v>3.506</v>
+        <v>3.725</v>
       </c>
       <c r="G43" s="1">
-        <v>3.705</v>
+        <v>3.949</v>
       </c>
       <c r="H43" s="1">
-        <v>3.699</v>
+        <v>3.948</v>
       </c>
       <c r="I43" s="1">
-        <v>3.54</v>
+        <v>3.798</v>
       </c>
       <c r="J43" s="1">
-        <v>3.196</v>
+        <v>3.44</v>
       </c>
       <c r="K43" s="1">
-        <v>2.624</v>
+        <v>2.825</v>
       </c>
       <c r="L43" s="1">
-        <v>1.905</v>
+        <v>2.026</v>
       </c>
       <c r="M43" s="1">
-        <v>1.142</v>
+        <v>1.205</v>
       </c>
       <c r="N43" s="1">
-        <v>0.409</v>
+        <v>0.423</v>
       </c>
       <c r="O43" s="1">
-        <v>-0.167</v>
+        <v>-0.192</v>
       </c>
       <c r="P43" s="1">
-        <v>-0.466</v>
+        <v>-0.48</v>
       </c>
       <c r="Q43" s="1">
-        <v>-0.5620000000000001</v>
+        <v>-0.573</v>
       </c>
       <c r="R43" s="1">
-        <v>-0.644</v>
+        <v>-0.665</v>
       </c>
       <c r="S43" s="1">
-        <v>-0.8090000000000001</v>
+        <v>-0.8</v>
       </c>
       <c r="T43" s="1">
-        <v>-0.993</v>
+        <v>-0.961</v>
       </c>
       <c r="U43" s="1">
-        <v>-1.023</v>
+        <v>-1.005</v>
       </c>
     </row>
     <row r="44" spans="1:21">
@@ -3329,61 +3332,126 @@
         <v>2.085</v>
       </c>
       <c r="C44" s="1">
-        <v>2.565</v>
+        <v>2.586</v>
       </c>
       <c r="D44" s="1">
-        <v>3.451</v>
+        <v>3.515</v>
       </c>
       <c r="E44" s="1">
-        <v>4.151</v>
+        <v>4.23</v>
       </c>
       <c r="F44" s="1">
-        <v>4.449</v>
+        <v>4.509</v>
       </c>
       <c r="G44" s="1">
-        <v>4.458</v>
+        <v>4.492</v>
       </c>
       <c r="H44" s="1">
-        <v>4.312</v>
+        <v>4.334</v>
       </c>
       <c r="I44" s="1">
-        <v>3.936</v>
+        <v>3.979</v>
       </c>
       <c r="J44" s="1">
-        <v>3.218</v>
+        <v>3.278</v>
       </c>
       <c r="K44" s="1">
-        <v>2.279</v>
+        <v>2.322</v>
       </c>
       <c r="L44" s="1">
-        <v>1.313</v>
+        <v>1.348</v>
       </c>
       <c r="M44" s="1">
-        <v>0.395</v>
+        <v>0.43</v>
       </c>
       <c r="N44" s="1">
-        <v>-0.314</v>
+        <v>-0.264</v>
       </c>
       <c r="O44" s="1">
-        <v>-0.65</v>
+        <v>-0.603</v>
       </c>
       <c r="P44" s="1">
-        <v>-0.742</v>
+        <v>-0.716</v>
       </c>
       <c r="Q44" s="1">
-        <v>-0.8100000000000001</v>
+        <v>-0.8179999999999999</v>
       </c>
       <c r="R44" s="1">
-        <v>-0.995</v>
+        <v>-1.017</v>
       </c>
       <c r="S44" s="1">
-        <v>-1.233</v>
+        <v>-1.235</v>
       </c>
       <c r="T44" s="1">
-        <v>-1.273</v>
+        <v>-1.281</v>
       </c>
       <c r="U44" s="1">
-        <v>-1.085</v>
+        <v>-1.098</v>
+      </c>
+    </row>
+    <row r="45" spans="1:21">
+      <c r="A45" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B45" s="1">
+        <v>2.695</v>
+      </c>
+      <c r="C45" s="1">
+        <v>3.194</v>
+      </c>
+      <c r="D45" s="1">
+        <v>3.949</v>
+      </c>
+      <c r="E45" s="1">
+        <v>4.276</v>
+      </c>
+      <c r="F45" s="1">
+        <v>4.323</v>
+      </c>
+      <c r="G45" s="1">
+        <v>4.254</v>
+      </c>
+      <c r="H45" s="1">
+        <v>3.968</v>
+      </c>
+      <c r="I45" s="1">
+        <v>3.295</v>
+      </c>
+      <c r="J45" s="1">
+        <v>2.354</v>
+      </c>
+      <c r="K45" s="1">
+        <v>1.386</v>
+      </c>
+      <c r="L45" s="1">
+        <v>0.489</v>
+      </c>
+      <c r="M45" s="1">
+        <v>-0.2</v>
+      </c>
+      <c r="N45" s="1">
+        <v>-0.5610000000000001</v>
+      </c>
+      <c r="O45" s="1">
+        <v>-0.6870000000000001</v>
+      </c>
+      <c r="P45" s="1">
+        <v>-0.757</v>
+      </c>
+      <c r="Q45" s="1">
+        <v>-0.902</v>
+      </c>
+      <c r="R45" s="1">
+        <v>-1.118</v>
+      </c>
+      <c r="S45" s="1">
+        <v>-1.174</v>
+      </c>
+      <c r="T45" s="1">
+        <v>-0.994</v>
+      </c>
+      <c r="U45" s="1">
+        <v>-0.763</v>
       </c>
     </row>
   </sheetData>
@@ -3398,22 +3466,22 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>